<commit_message>
Weekly update for 07.06.26
</commit_message>
<xml_diff>
--- a/jdca_weekly_metrics_asof_2026-07-06.xlsx
+++ b/jdca_weekly_metrics_asof_2026-07-06.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>1-Week Return (Past 5 Trading Days)</t>
+          <t>1-Week Return (Snapshot-Anchored)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -570,7 +570,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1099864866816</v>
+        <v>1092543774720</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -587,13 +587,13 @@
         <v>1238</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006671470181780825</v>
+        <v>-0.0242859299413527</v>
       </c>
       <c r="M2" t="n">
-        <v>-3.161159215083831</v>
+        <v>-4.922605191041018</v>
       </c>
       <c r="N2" t="n">
-        <v>-4.910313607815119</v>
+        <v>-5.337069499005787</v>
       </c>
       <c r="O2" t="n">
         <v>0.1204564938752037</v>
@@ -608,17 +608,17 @@
         <v>0.9962829505225028</v>
       </c>
       <c r="S2" t="n">
-        <v>28.2</v>
+        <v>28.17</v>
       </c>
       <c r="T2" t="n">
-        <v>43.737232</v>
+        <v>43.49237</v>
       </c>
       <c r="U2" t="n">
         <v>1.497</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>[[1747368000000, 752.0698], [1747972800000, 708.6967], [1748577600000, 732.4884], [1749182400000, 764.4721], [1749787200000, 813.6046], [1750392000000, 757.3723], [1750996800000, 770.0031], [1751601600000, 775.1863], [1752206400000, 787.4396], [1752811200000, 766.2893], [1753416000000, 806.9814], [1754020800000, 756.9752], [1754625600000, 621.2553], [1755230400000, 697.8337], [1755835200000, 708.233], [1756440000000, 729.0319], [1757044800000, 723.6879], [1757649600000, 751.7314], [1758254400000, 748.3478], [1758859200000, 721.0308], [1759464000000, 835.8022], [1760068800000, 829.4531], [1760673600000, 798.9417], [1761278400000, 821.4521], [1761883200000, 858.6808], [1762491600000, 919.8929], [1763096400000, 1021.8127], [1763701200000, 1056.1162], [1764306000000, 1071.8329], [1764910800000, 1006.8932], [1765515600000, 1024.0352], [1766120400000, 1067.8165], [1766725200000, 1074.1052], [1767330000000, 1076.7064], [1767934800000, 1059.9633], [1768539600000, 1034.8883], [1769144400000, 1060.6908], [1769749200000, 1033.6425], [1770354000000, 1054.6014], [1770958800000, 1038.2128], [1771563600000, 1007.7852], [1772168400000, 1050.1821], [1772773200000, 988.6282], [1773374400000, 983.3872], [1773979200000, 905.1419], [1774584000000, 876.7308], [1775188800000, 933.9722], [1775793600000, 937.8555], [1776398400000, 925.437], [1777003200000, 882.441], [1777608000000, 961.6746], [1778212800000, 946.8201], [1778817600000, 1004.92], [1779422400000, 1065.0], [1780027200000, 1105.0], [1780632000000, 1131.42], [1781236800000, 1133.0], [1781841600000, 1098.5699], [1782446400000, 1208.12], [1783051200000, 1213.91], [1783656000000, 1200.0601]]</t>
+          <t>[[1747368000000, 752.0698], [1747972800000, 708.6967], [1748577600000, 732.4883], [1749182400000, 764.4721], [1749787200000, 813.6046], [1750392000000, 757.3723], [1750996800000, 770.0029], [1751601600000, 775.1863], [1752206400000, 787.4397], [1752811200000, 766.2892], [1753416000000, 806.9814], [1754020800000, 756.9752], [1754625600000, 621.2553], [1755230400000, 697.8337], [1755835200000, 708.2331], [1756440000000, 729.0319], [1757044800000, 723.6879], [1757649600000, 751.7314], [1758254400000, 748.3479], [1758859200000, 721.0308], [1759464000000, 835.8022], [1760068800000, 829.4531], [1760673600000, 798.9417], [1761278400000, 821.4521], [1761883200000, 858.6808], [1762491600000, 919.8929], [1763096400000, 1021.8127], [1763701200000, 1056.1162], [1764306000000, 1071.8329], [1764910800000, 1006.8933], [1765515600000, 1024.0352], [1766120400000, 1067.8165], [1766725200000, 1074.1052], [1767330000000, 1076.7063], [1767934800000, 1059.9634], [1768539600000, 1034.8883], [1769144400000, 1060.6908], [1769749200000, 1033.6426], [1770354000000, 1054.6014], [1770958800000, 1038.2128], [1771563600000, 1007.7852], [1772168400000, 1050.1821], [1772773200000, 988.6282], [1773374400000, 983.3872], [1773979200000, 905.1419], [1774584000000, 876.7308], [1775188800000, 933.9722], [1775793600000, 937.8555], [1776398400000, 925.437], [1777003200000, 882.441], [1777608000000, 961.6746], [1778212800000, 946.8201], [1778817600000, 1004.92], [1779422400000, 1065.0], [1780027200000, 1105.0], [1780632000000, 1131.42], [1781236800000, 1133.0], [1781841600000, 1098.5699], [1782446400000, 1208.12], [1783051200000, 1213.91], [1783656000000, 1200.0601]]</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>218718126080</v>
+        <v>217855295488</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -669,13 +669,13 @@
         <v>68.48814681010441</v>
       </c>
       <c r="L3" t="n">
-        <v>0.02475553638992656</v>
+        <v>0.01903181973606305</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.01845855791309248</v>
+        <v>-0.5908302232994433</v>
       </c>
       <c r="N3" t="n">
-        <v>-1.767612950644382</v>
+        <v>-1.005294531264211</v>
       </c>
       <c r="O3" t="n">
         <v>0.00366748802874417</v>
@@ -690,10 +690,10 @@
         <v>0.6134622583629368</v>
       </c>
       <c r="S3" t="n">
-        <v>4.17</v>
+        <v>4.16</v>
       </c>
       <c r="T3" t="n">
-        <v>11.853717</v>
+        <v>11.835337</v>
       </c>
       <c r="U3" t="n">
         <v>0.788</v>
@@ -734,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>103111598080</v>
+        <v>102991912960</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -751,13 +751,13 @@
         <v>49.91109967191108</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007916185018587263</v>
+        <v>-0.01888095070371199</v>
       </c>
       <c r="M4" t="n">
-        <v>-3.285630698764475</v>
+        <v>-4.382107267276947</v>
       </c>
       <c r="N4" t="n">
-        <v>-5.034785091495763</v>
+        <v>-4.796571575241715</v>
       </c>
       <c r="O4" t="n">
         <v>-0.07193850874637009</v>
@@ -772,10 +772,10 @@
         <v>1.024577649793844</v>
       </c>
       <c r="S4" t="n">
-        <v>2.25</v>
+        <v>2.26</v>
       </c>
       <c r="T4" t="n">
-        <v>19.144445</v>
+        <v>19.037611</v>
       </c>
       <c r="U4" t="n">
         <v>1.005</v>
@@ -816,7 +816,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>132928053248</v>
+        <v>129204731904</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -833,13 +833,13 @@
         <v>529.989990234375</v>
       </c>
       <c r="L5" t="n">
-        <v>0.07784839582095393</v>
+        <v>0.05992201205787917</v>
       </c>
       <c r="M5" t="n">
-        <v>5.290827385189645</v>
+        <v>3.498189008882169</v>
       </c>
       <c r="N5" t="n">
-        <v>3.541672992458356</v>
+        <v>3.083724700917401</v>
       </c>
       <c r="O5" t="n">
         <v>0.1681446178907759</v>
@@ -854,10 +854,10 @@
         <v>1.182815494631559</v>
       </c>
       <c r="S5" t="n">
-        <v>16.84</v>
+        <v>16.87</v>
       </c>
       <c r="T5" t="n">
-        <v>31.100948</v>
+        <v>30.17605</v>
       </c>
       <c r="U5" t="n">
         <v>3.023</v>
@@ -898,7 +898,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>37354401792</v>
+        <v>36091715584</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -915,13 +915,13 @@
         <v>37.52000045776367</v>
       </c>
       <c r="L6" t="n">
-        <v>0.06753172886558145</v>
+        <v>0.06283027901832572</v>
       </c>
       <c r="M6" t="n">
-        <v>4.259160689652397</v>
+        <v>3.789015704926824</v>
       </c>
       <c r="N6" t="n">
-        <v>2.510006296921108</v>
+        <v>3.374551396962056</v>
       </c>
       <c r="O6" t="n">
         <v>0.2777974182995997</v>
@@ -939,7 +939,7 @@
         <v>2.12</v>
       </c>
       <c r="T6" t="n">
-        <v>16.745283</v>
+        <v>16.179245</v>
       </c>
       <c r="U6" t="n">
         <v>2.332</v>
@@ -980,7 +980,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5939577856</v>
+        <v>5799730176</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -997,13 +997,13 @@
         <v>78.48000335693359</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1269118982717725</v>
+        <v>0.09831412716136301</v>
       </c>
       <c r="M7" t="n">
-        <v>10.1971776302715</v>
+        <v>7.337400519230552</v>
       </c>
       <c r="N7" t="n">
-        <v>8.448023237540214</v>
+        <v>6.922936211265784</v>
       </c>
       <c r="O7" t="n">
         <v>0.1802059689247653</v>
@@ -1060,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>1147952768</v>
+        <v>1099251712</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1077,13 +1077,13 @@
         <v>6.550000190734863</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1608186959201146</v>
+        <v>0.1507246300693923</v>
       </c>
       <c r="M8" t="n">
-        <v>13.58785739510571</v>
+        <v>12.57845081003348</v>
       </c>
       <c r="N8" t="n">
-        <v>11.83870300237442</v>
+        <v>12.16398650206871</v>
       </c>
       <c r="O8" t="n">
         <v>-0.02457005868142936</v>
@@ -1140,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>1009373440</v>
+        <v>978543168</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1157,13 +1157,13 @@
         <v>4.420000076293945</v>
       </c>
       <c r="L9" t="n">
-        <v>0.06569345479222655</v>
+        <v>0.04285718786473258</v>
       </c>
       <c r="M9" t="n">
-        <v>4.075333282316906</v>
+        <v>1.79170658956751</v>
       </c>
       <c r="N9" t="n">
-        <v>2.326178889585617</v>
+        <v>1.377242281602742</v>
       </c>
       <c r="O9" t="n">
         <v>-0.05194800369332064</v>
@@ -1237,13 +1237,13 @@
         <v>2.089999914169312</v>
       </c>
       <c r="L10" t="n">
-        <v>0.03906255675247072</v>
+        <v>-0.01481480042466765</v>
       </c>
       <c r="M10" t="n">
-        <v>1.412243478341324</v>
+        <v>-3.975492239372513</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.3369109143899651</v>
+        <v>-4.389956547337281</v>
       </c>
       <c r="O10" t="n">
         <v>-0.2035927682075241</v>
@@ -1300,7 +1300,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>213014144</v>
+        <v>202336464</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1317,13 +1317,13 @@
         <v>2.839999914169312</v>
       </c>
       <c r="L11" t="n">
-        <v>0.087447160776007</v>
+        <v>-0.03504380008766883</v>
       </c>
       <c r="M11" t="n">
-        <v>6.250703880694952</v>
+        <v>-5.998392205672632</v>
       </c>
       <c r="N11" t="n">
-        <v>4.501549487963663</v>
+        <v>-6.412856513637399</v>
       </c>
       <c r="O11" t="n">
         <v>-0.1977107103217441</v>
@@ -1380,7 +1380,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>6537751</v>
+        <v>5938940</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1397,13 +1397,13 @@
         <v>55</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2545454260841</v>
+        <v>0.2297029658563345</v>
       </c>
       <c r="M12" t="n">
-        <v>22.96053041150425</v>
+        <v>20.47628438872771</v>
       </c>
       <c r="N12" t="n">
-        <v>21.21137601877297</v>
+        <v>20.06182008076294</v>
       </c>
       <c r="O12" t="n">
         <v>-0.6451428617749895</v>
@@ -1460,7 +1460,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>411208960</v>
+        <v>435556864</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1477,13 +1477,13 @@
         <v>3.039999961853027</v>
       </c>
       <c r="L13" t="n">
-        <v>0.03448282949422898</v>
+        <v>-0.004149373488428587</v>
       </c>
       <c r="M13" t="n">
-        <v>0.9542707525171501</v>
+        <v>-2.908949545748607</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.794883640214139</v>
+        <v>-3.323413853713375</v>
       </c>
       <c r="O13" t="n">
         <v>1.412060385794805</v>
@@ -1498,7 +1498,7 @@
         <v>1.597154168340123</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.14</v>
+        <v>-1.1</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="n">
@@ -1540,7 +1540,7 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>295916032</v>
+        <v>295533728</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1557,13 +1557,13 @@
         <v>6.599999904632568</v>
       </c>
       <c r="L14" t="n">
-        <v>0.03157898039038542</v>
+        <v>0.005128200112166637</v>
       </c>
       <c r="M14" t="n">
-        <v>0.6638858421327942</v>
+        <v>-1.981192185689085</v>
       </c>
       <c r="N14" t="n">
-        <v>-1.085268550598495</v>
+        <v>-2.395656493653853</v>
       </c>
       <c r="O14" t="n">
         <v>0.04812835997278464</v>
@@ -1620,7 +1620,7 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>33987824</v>
+        <v>38519532</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1637,13 +1637,13 @@
         <v>0.1599999964237213</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>-0.09999997764825841</v>
       </c>
       <c r="M15" t="n">
-        <v>-2.494012196905748</v>
+        <v>-12.49400996173159</v>
       </c>
       <c r="N15" t="n">
-        <v>-4.243166589637037</v>
+        <v>-12.90847426969636</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -1700,7 +1700,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>21373968</v>
+        <v>22719934</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1717,13 +1717,13 @@
         <v>28.03000068664551</v>
       </c>
       <c r="L16" t="n">
-        <v>0.07280215902427067</v>
+        <v>0.05826555849195914</v>
       </c>
       <c r="M16" t="n">
-        <v>4.786203705521319</v>
+        <v>3.332543652290165</v>
       </c>
       <c r="N16" t="n">
-        <v>3.03704931279003</v>
+        <v>2.918079344325397</v>
       </c>
       <c r="O16" t="n">
         <v>1.055263168626875</v>
@@ -1780,7 +1780,7 @@
         <v>0.1037318632006645</v>
       </c>
       <c r="G17" t="n">
-        <v>5129883.780276328</v>
+        <v>4901889.028582871</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1797,13 +1797,13 @@
         <v>6.970780890520132</v>
       </c>
       <c r="L17" t="n">
-        <v>0.2695034846988034</v>
+        <v>0.2819493734216099</v>
       </c>
       <c r="M17" t="n">
-        <v>24.45633627297459</v>
+        <v>25.70092514525524</v>
       </c>
       <c r="N17" t="n">
-        <v>22.7071818802433</v>
+        <v>25.28646083729047</v>
       </c>
       <c r="O17" t="n">
         <v>2.579999923706055</v>
@@ -1821,7 +1821,7 @@
         <v>678.84</v>
       </c>
       <c r="T17" t="n">
-        <v>0.05303164</v>
+        <v>0.05067468</v>
       </c>
       <c r="U17" t="n">
         <v>1.334</v>
@@ -1862,7 +1862,7 @@
         <v>0.1037318632006645</v>
       </c>
       <c r="G18" t="n">
-        <v>11762989.14264858</v>
+        <v>11670549.11514848</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1879,13 +1879,13 @@
         <v>0.1850576480059685</v>
       </c>
       <c r="L18" t="n">
-        <v>0.00603619944721201</v>
+        <v>0.01589912203100141</v>
       </c>
       <c r="M18" t="n">
-        <v>-1.890392252184547</v>
+        <v>-0.9040999938056071</v>
       </c>
       <c r="N18" t="n">
-        <v>-3.639546644915836</v>
+        <v>-1.318564301770375</v>
       </c>
       <c r="O18" t="n">
         <v>0.3679890444869984</v>
@@ -1942,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>1673477504</v>
+        <v>1681107200</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1959,13 +1959,13 @@
         <v>40.71500015258789</v>
       </c>
       <c r="L19" t="n">
-        <v>0.03432647027522462</v>
+        <v>0.04996714181300055</v>
       </c>
       <c r="M19" t="n">
-        <v>0.9386348306167136</v>
+        <v>2.502701984394307</v>
       </c>
       <c r="N19" t="n">
-        <v>-0.8105195621145755</v>
+        <v>2.088237676429539</v>
       </c>
       <c r="O19" t="n">
         <v>-0.07980405138224811</v>
@@ -2022,7 +2022,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>3881501</v>
+        <v>3636782</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2039,13 +2039,13 @@
         <v>6.25</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.0416667246156246</v>
+        <v>0.4194026293138329</v>
       </c>
       <c r="M20" t="n">
-        <v>-6.660684658468208</v>
+        <v>39.44625073447754</v>
       </c>
       <c r="N20" t="n">
-        <v>-8.409839051199498</v>
+        <v>39.03178642651277</v>
       </c>
       <c r="O20" t="n">
         <v>-0.4132653297061272</v>
@@ -2102,7 +2102,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>305277824</v>
+        <v>307207552</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2119,13 +2119,13 @@
         <v>4.599999904632568</v>
       </c>
       <c r="L21" t="n">
-        <v>0.05026456578268257</v>
+        <v>0.02319585348318465</v>
       </c>
       <c r="M21" t="n">
-        <v>2.532444381362509</v>
+        <v>-0.1744268485872835</v>
       </c>
       <c r="N21" t="n">
-        <v>0.7832899886312195</v>
+        <v>-0.5888911565520516</v>
       </c>
       <c r="O21" t="n">
         <v>1.629139108399771</v>
@@ -2182,7 +2182,7 @@
         <v>1.143772125244141</v>
       </c>
       <c r="G22" t="n">
-        <v>89785370.66732788</v>
+        <v>86257272.8694458</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2199,13 +2199,13 @@
         <v>14.1827739167129</v>
       </c>
       <c r="L22" t="n">
-        <v>0.04135899301190538</v>
+        <v>0.04612324943834278</v>
       </c>
       <c r="M22" t="n">
-        <v>1.641887104284789</v>
+        <v>2.11831274692853</v>
       </c>
       <c r="N22" t="n">
-        <v>-0.1072672884464998</v>
+        <v>1.703848438963762</v>
       </c>
       <c r="O22" t="n">
         <v>-0.3686566955981097</v>

</xml_diff>

<commit_message>
Weekly update for July 6, 2026
</commit_message>
<xml_diff>
--- a/jdca_weekly_metrics_asof_2026-07-06.xlsx
+++ b/jdca_weekly_metrics_asof_2026-07-06.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:W22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,40 +501,45 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>QTD Return</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Total Return (YTD)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Average Daily Volume (100D)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Avg Daily Volume (Last 5 Days)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Relative Volume (Last 5D vs 100D)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>EPS (Basic)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>P/E (Trailing)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Current Ratio</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Weekly History (USD)</t>
         </is>
@@ -570,7 +575,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1088669024256</v>
+        <v>1084959490048</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -587,38 +592,41 @@
         <v>1238</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.006671470181780825</v>
+        <v>-0.02428592994135226</v>
       </c>
       <c r="M2" t="n">
-        <v>-3.161159215083831</v>
+        <v>-3.732281056631082</v>
       </c>
       <c r="N2" t="n">
-        <v>-4.910313607815119</v>
+        <v>-5.337073139418136</v>
       </c>
       <c r="O2" t="n">
+        <v>0.0005252535409325798</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.1204564938752037</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>3166490</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>3154720</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>0.9962829505225028</v>
       </c>
-      <c r="S2" t="n">
-        <v>28.17</v>
-      </c>
       <c r="T2" t="n">
-        <v>43.338123</v>
+        <v>28.21</v>
       </c>
       <c r="U2" t="n">
+        <v>43.12921</v>
+      </c>
+      <c r="V2" t="n">
         <v>1.497</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>[[1747368000000, 752.0698], [1747972800000, 708.6967], [1748577600000, 732.4884], [1749182400000, 764.4721], [1749787200000, 813.6046], [1750392000000, 757.3723], [1750996800000, 770.0031], [1751601600000, 775.1863], [1752206400000, 787.4397], [1752811200000, 766.2892], [1753416000000, 806.9814], [1754020800000, 756.9751], [1754625600000, 621.2552], [1755230400000, 697.8337], [1755835200000, 708.233], [1756440000000, 729.0319], [1757044800000, 723.6879], [1757649600000, 751.7314], [1758254400000, 748.3478], [1758859200000, 721.0308], [1759464000000, 835.8022], [1760068800000, 829.4531], [1760673600000, 798.9417], [1761278400000, 821.4521], [1761883200000, 858.6808], [1762491600000, 919.8929], [1763096400000, 1021.8127], [1763701200000, 1056.1162], [1764306000000, 1071.8329], [1764910800000, 1006.8932], [1765515600000, 1024.0352], [1766120400000, 1067.8165], [1766725200000, 1074.1052], [1767330000000, 1076.7064], [1767934800000, 1059.9633], [1768539600000, 1034.8883], [1769144400000, 1060.6908], [1769749200000, 1033.6425], [1770354000000, 1054.6014], [1770958800000, 1038.2128], [1771563600000, 1007.7852], [1772168400000, 1050.1821], [1772773200000, 988.6282], [1773374400000, 983.3872], [1773979200000, 905.1419], [1774584000000, 876.7308], [1775188800000, 933.9722], [1775793600000, 937.8555], [1776398400000, 925.437], [1777003200000, 882.441], [1777608000000, 961.6746], [1778212800000, 946.8201], [1778817600000, 1004.92], [1779422400000, 1065.0], [1780027200000, 1105.0], [1780632000000, 1131.42], [1781236800000, 1133.0], [1781841600000, 1098.5699], [1782446400000, 1208.12], [1783051200000, 1213.91], [1783656000000, 1200.0601]]</t>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>[[1747368000000, 752.0698], [1747972800000, 708.6967], [1748577600000, 732.4883], [1749182400000, 764.4721], [1749787200000, 813.6046], [1750392000000, 757.3723], [1750996800000, 770.003], [1751601600000, 775.1863], [1752206400000, 787.4396], [1752811200000, 766.2892], [1753416000000, 806.9814], [1754020800000, 756.9752], [1754625600000, 621.2552], [1755230400000, 697.8337], [1755835200000, 708.2331], [1756440000000, 729.0319], [1757044800000, 723.6879], [1757649600000, 751.7314], [1758254400000, 748.3479], [1758859200000, 721.0308], [1759464000000, 835.8022], [1760068800000, 829.4531], [1760673600000, 798.9417], [1761278400000, 821.4521], [1761883200000, 858.6808], [1762491600000, 919.8929], [1763096400000, 1021.8127], [1763701200000, 1056.1162], [1764306000000, 1071.8329], [1764910800000, 1006.8933], [1765515600000, 1024.0352], [1766120400000, 1067.8165], [1766725200000, 1074.1052], [1767330000000, 1076.7063], [1767934800000, 1059.9634], [1768539600000, 1034.8883], [1769144400000, 1060.6908], [1769749200000, 1033.6426], [1770354000000, 1054.6014], [1770958800000, 1038.2128], [1771563600000, 1007.7852], [1772168400000, 1050.1821], [1772773200000, 988.6282], [1773374400000, 983.3872], [1773979200000, 905.1419], [1774584000000, 876.7308], [1775188800000, 933.9722], [1775793600000, 937.8555], [1776398400000, 925.437], [1777003200000, 882.441], [1777608000000, 961.6746], [1778212800000, 946.8201], [1778817600000, 1004.92], [1779422400000, 1065.0], [1780027200000, 1105.0], [1780632000000, 1131.42], [1781236800000, 1133.0], [1781841600000, 1098.5699], [1782446400000, 1208.12], [1783051200000, 1213.91], [1783656000000, 1200.0601]]</t>
         </is>
       </c>
     </row>
@@ -652,7 +660,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>217611927552</v>
+        <v>216581390336</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -669,36 +677,39 @@
         <v>68.48814681010441</v>
       </c>
       <c r="L3" t="n">
-        <v>0.02475553638992656</v>
+        <v>0.01903181973606305</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.01845855791309248</v>
+        <v>0.5994939111104491</v>
       </c>
       <c r="N3" t="n">
-        <v>-1.767612950644382</v>
+        <v>-1.005298171676605</v>
       </c>
       <c r="O3" t="n">
+        <v>0.02753441244549393</v>
+      </c>
+      <c r="P3" t="n">
         <v>0.00366748802874417</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>17459656</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>10710840</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>0.6134622583629368</v>
       </c>
-      <c r="S3" t="n">
-        <v>4.16</v>
-      </c>
       <c r="T3" t="n">
-        <v>11.822116</v>
+        <v>4.17</v>
       </c>
       <c r="U3" t="n">
+        <v>11.737914</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.788</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>[[1747368000000, 61.4009], [1747972800000, 64.2434], [1748577600000, 68.202], [1749182400000, 71.1876], [1749787200000, 76.1478], [1750392000000, 70.3673], [1750996800000, 65.3499], [1751601600000, 65.9795], [1752206400000, 65.7505], [1752811200000, 61.3436], [1753416000000, 68.3928], [1754020800000, 45.9672], [1754625600000, 48.7239], [1755230400000, 49.9925], [1755835200000, 54.9642], [1756440000000, 54.4626], [1757044800000, 53.2761], [1757649600000, 52.9288], [1758254400000, 59.2278], [1758859200000, 53.6427], [1759464000000, 57.5204], [1760068800000, 54.916], [1760673600000, 52.4465], [1761278400000, 51.0864], [1761883200000, 47.7102], [1762491600000, 44.064], [1763096400000, 46.5527], [1763701200000, 45.945], [1764306000000, 47.6041], [1764910800000, 46.1668], [1765515600000, 48.4048], [1766120400000, 46.3887], [1766725200000, 50.5462], [1767330000000, 50.5366], [1767934800000, 56.7295], [1768539600000, 60.1249], [1769144400000, 60.0574], [1769749200000, 57.3275], [1770354000000, 45.9546], [1770958800000, 47.8163], [1771563600000, 45.7424], [1772168400000, 36.1251], [1772773200000, 37.2151], [1773374400000, 36.6171], [1773979200000, 35.2377], [1774584000000, 34.765], [1775188800000, 36.98], [1775793600000, 37.52], [1776398400000, 40.52], [1777003200000, 41.17], [1777608000000, 43.88], [1778212800000, 46.07], [1778817600000, 44.74], [1779422400000, 44.96], [1780027200000, 45.58], [1780632000000, 42.96], [1781236800000, 43.88], [1781841600000, 43.19], [1782446400000, 48.07], [1783051200000, 50.43], [1783656000000, 49.26]]</t>
         </is>
@@ -734,7 +745,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>102944038912</v>
+        <v>105036193792</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -751,36 +762,39 @@
         <v>49.91109967191108</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.007916185018587263</v>
+        <v>-0.01888095070371199</v>
       </c>
       <c r="M4" t="n">
-        <v>-3.285630698764475</v>
+        <v>-3.191783132867054</v>
       </c>
       <c r="N4" t="n">
-        <v>-5.034785091495763</v>
+        <v>-4.796575215654109</v>
       </c>
       <c r="O4" t="n">
+        <v>-0.001172040254087792</v>
+      </c>
+      <c r="P4" t="n">
         <v>-0.07193850874637009</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>3618857</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>3707800</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>1.024577649793844</v>
       </c>
-      <c r="S4" t="n">
-        <v>2.26</v>
-      </c>
       <c r="T4" t="n">
-        <v>19.02876</v>
+        <v>2.25</v>
       </c>
       <c r="U4" t="n">
+        <v>19.501778</v>
+      </c>
+      <c r="V4" t="n">
         <v>1.005</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>[[1747368000000, 48.9637], [1747972800000, 49.2479], [1748577600000, 46.7751], [1749182400000, 47.8173], [1749787200000, 47.0593], [1750392000000, 45.3444], [1750996800000, 45.335], [1751601600000, 45.7613], [1752206400000, 46.055], [1752811200000, 45.7803], [1753416000000, 47.7225], [1754020800000, 44.2928], [1754625600000, 44.6528], [1755230400000, 47.1541], [1755835200000, 48.651], [1756440000000, 46.8793], [1757044800000, 44.0559], [1757649600000, 44.5581], [1758254400000, 45.136], [1758859200000, 43.1464], [1759464000000, 48.2247], [1760068800000, 45.5624], [1760673600000, 47.9594], [1761278400000, 48.9258], [1761883200000, 47.9215], [1762491600000, 47.0498], [1763096400000, 49.3995], [1763701200000, 47.0214], [1764306000000, 47.2583], [1764910800000, 46.9267], [1765515600000, 46.1213], [1766120400000, 45.6476], [1766725200000, 45.9224], [1767330000000, 45.695], [1767934800000, 46.4529], [1768539600000, 44.1412], [1769144400000, 44.7191], [1769749200000, 44.5675], [1770354000000, 45.316], [1770958800000, 43.5917], [1771563600000, 44.3023], [1772168400000, 46.1024], [1772773200000, 42.2084], [1773374400000, 41.3083], [1773979200000, 42.2558], [1774584000000, 44.3212], [1775188800000, 45.3729], [1775793600000, 44.3023], [1776398400000, 45.5339], [1777003200000, 44.3212], [1777608000000, 43.658], [1778212800000, 43.31], [1778817600000, 42.69], [1779422400000, 44.29], [1780027200000, 43.67], [1780632000000, 45.02], [1781236800000, 44.25], [1781841600000, 42.38], [1782446400000, 42.95], [1783051200000, 43.16], [1783656000000, 42.61]]</t>
         </is>
@@ -816,7 +830,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>127110832128</v>
+        <v>123450957824</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -833,36 +847,39 @@
         <v>529.989990234375</v>
       </c>
       <c r="L5" t="n">
-        <v>0.07784839582095393</v>
+        <v>0.05992201205787917</v>
       </c>
       <c r="M5" t="n">
-        <v>5.290827385189645</v>
+        <v>4.688513143292061</v>
       </c>
       <c r="N5" t="n">
-        <v>3.541672992458356</v>
+        <v>3.083721060505007</v>
       </c>
       <c r="O5" t="n">
+        <v>0.06615266873827985</v>
+      </c>
+      <c r="P5" t="n">
         <v>0.1681446178907759</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>1455730</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>1721860</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>1.182815494631559</v>
       </c>
-      <c r="S5" t="n">
-        <v>16.87</v>
-      </c>
       <c r="T5" t="n">
-        <v>29.687017</v>
+        <v>16.85</v>
       </c>
       <c r="U5" t="n">
+        <v>28.866468</v>
+      </c>
+      <c r="V5" t="n">
         <v>3.023</v>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>[[1747368000000, 438.65], [1747972800000, 436.0], [1748577600000, 442.05], [1749182400000, 450.5], [1749787200000, 455.45], [1750392000000, 440.87], [1750996800000, 441.3], [1751601600000, 459.62], [1752206400000, 468.85], [1752811200000, 459.81], [1753416000000, 469.65], [1754020800000, 462.13], [1754625600000, 366.54], [1755230400000, 392.79], [1755835200000, 395.12], [1756440000000, 391.02], [1757044800000, 396.12], [1757649600000, 394.53], [1758254400000, 383.12], [1758859200000, 385.74], [1759464000000, 403.3], [1760068800000, 407.79], [1760673600000, 416.81], [1761278400000, 421.39], [1761883200000, 425.57], [1762491600000, 409.47], [1763096400000, 437.15], [1763701200000, 426.76], [1764306000000, 433.61], [1764910800000, 455.48], [1765515600000, 452.04], [1766120400000, 456.2], [1766725200000, 462.9], [1767330000000, 452.13], [1767934800000, 463.86], [1768539600000, 441.36], [1769144400000, 468.41], [1769749200000, 469.9], [1770354000000, 477.92], [1770958800000, 491.47], [1771563600000, 476.9], [1772168400000, 496.83], [1772773200000, 456.69], [1773374400000, 469.34], [1773979200000, 454.0], [1774584000000, 433.07], [1775188800000, 438.71], [1775793600000, 436.27], [1776398400000, 441.2], [1777003200000, 430.29], [1777608000000, 423.92], [1778212800000, 429.82], [1778817600000, 436.95], [1779422400000, 434.52], [1780027200000, 447.54], [1780632000000, 446.83], [1781236800000, 444.93], [1781841600000, 451.63], [1782446400000, 491.34], [1783051200000, 528.04], [1783656000000, 529.59]]</t>
         </is>
@@ -898,7 +915,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>36144328704</v>
+        <v>36018061312</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -915,36 +932,39 @@
         <v>37.52000045776367</v>
       </c>
       <c r="L6" t="n">
-        <v>0.06753172886558145</v>
+        <v>0.06283027901832594</v>
       </c>
       <c r="M6" t="n">
-        <v>4.259160689652397</v>
+        <v>4.979339839336738</v>
       </c>
       <c r="N6" t="n">
-        <v>2.510006296921108</v>
+        <v>3.374547756549684</v>
       </c>
       <c r="O6" t="n">
+        <v>0.08124257042691219</v>
+      </c>
+      <c r="P6" t="n">
         <v>0.2777974182995997</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>41439</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>44420</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>1.071937064118343</v>
       </c>
-      <c r="S6" t="n">
-        <v>2.12</v>
-      </c>
       <c r="T6" t="n">
-        <v>16.202831</v>
+        <v>2.05</v>
       </c>
       <c r="U6" t="n">
+        <v>16.697561</v>
+      </c>
+      <c r="V6" t="n">
         <v>2.332</v>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>[[1747368000000, 22.5342], [1747972800000, 22.9106], [1748577600000, 25.1095], [1749182400000, 25.5354], [1749787200000, 25.0501], [1750392000000, 23.6832], [1750996800000, 24.535], [1751601600000, 23.57], [1752206400000, 22.68], [1752811200000, 21.7], [1753416000000, 23.8], [1754020800000, 25.01], [1754625600000, 26.54], [1755230400000, 26.74], [1755835200000, 27.53], [1756440000000, 26.19], [1757044800000, 28.25], [1757649600000, 28.69], [1758254400000, 27.56], [1758859200000, 25.99], [1759464000000, 27.67], [1760068800000, 26.09], [1760673600000, 27.26], [1761278400000, 27.135], [1761883200000, 27.17], [1762491600000, 27.33], [1763096400000, 27.13], [1763701200000, 27.63], [1764306000000, 28.33], [1764910800000, 29.53], [1765515600000, 29.66], [1766120400000, 29.37], [1766725200000, 29.41], [1767330000000, 28.4], [1767934800000, 29.13], [1768539600000, 28.32], [1769144400000, 30.095], [1769749200000, 29.97], [1770354000000, 30.11], [1770958800000, 34.65], [1771563600000, 34.29], [1772168400000, 34.21], [1772773200000, 31.36], [1773374400000, 34.27], [1773979200000, 32.85], [1774584000000, 34.93], [1775188800000, 35.8], [1775793600000, 33.88], [1776398400000, 33.62], [1777003200000, 33.75], [1777608000000, 35.57], [1778212800000, 35.37], [1778817600000, 35.43], [1779422400000, 36.53], [1780027200000, 36.51], [1780632000000, 32.52], [1781236800000, 32.06], [1781841600000, 33.63], [1782446400000, 33.91], [1783051200000, 36.12], [1783656000000, 36.2]]</t>
         </is>
@@ -980,7 +1000,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5812040704</v>
+        <v>5642145792</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -997,34 +1017,37 @@
         <v>78.48000335693359</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1269118982717725</v>
+        <v>0.09831412716136279</v>
       </c>
       <c r="M7" t="n">
-        <v>10.1971776302715</v>
+        <v>8.527724653640423</v>
       </c>
       <c r="N7" t="n">
-        <v>8.448023237540214</v>
+        <v>6.922932570853368</v>
       </c>
       <c r="O7" t="n">
+        <v>0.1347634461082046</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.1802059689247653</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>1838433</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>1795200</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>0.9764837772167928</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>-6.17</v>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="n">
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="n">
         <v>17.965</v>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>[[1747368000000, 38.77], [1747972800000, 36.86], [1748577600000, 36.29], [1749182400000, 41.86], [1749787200000, 41.36], [1750392000000, 44.25], [1750996800000, 47.49], [1751601600000, 52.17], [1752206400000, 56.8], [1752811200000, 65.13], [1753416000000, 64.76], [1754020800000, 56.09], [1754625600000, 55.0], [1755230400000, 59.73], [1755835200000, 54.32], [1756440000000, 51.83], [1757044800000, 54.86], [1757649600000, 56.26], [1758254400000, 62.32], [1758859200000, 61.67], [1759464000000, 67.74], [1760068800000, 73.07], [1760673600000, 69.15], [1761278400000, 67.61], [1761883200000, 63.99], [1762491600000, 55.12], [1763096400000, 52.53], [1763701200000, 50.23], [1764306000000, 53.47], [1764910800000, 56.88], [1765515600000, 56.68], [1766120400000, 55.86], [1766725200000, 55.08], [1767330000000, 53.77], [1767934800000, 53.84], [1768539600000, 53.51], [1769144400000, 55.52], [1769749200000, 49.96], [1770354000000, 48.74], [1770958800000, 53.07], [1771563600000, 53.46], [1772168400000, 60.14], [1772773200000, 56.5], [1773374400000, 48.75], [1773979200000, 46.24], [1774584000000, 45.75], [1775188800000, 49.51], [1775793600000, 51.22], [1776398400000, 57.99], [1777003200000, 48.785], [1777608000000, 51.63], [1778212800000, 54.83], [1778817600000, 48.41], [1779422400000, 50.36], [1780027200000, 56.18], [1780632000000, 51.84], [1781236800000, 49.8], [1781841600000, 54.09], [1782446400000, 54.92], [1783051200000, 60.08], [1783656000000, 61.89]]</t>
         </is>
@@ -1060,7 +1083,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>1089511552</v>
+        <v>1074205440</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1077,34 +1100,37 @@
         <v>6.550000190734863</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1608186959201146</v>
+        <v>0.1507246300693923</v>
       </c>
       <c r="M8" t="n">
-        <v>13.58785739510571</v>
+        <v>13.76877494444337</v>
       </c>
       <c r="N8" t="n">
-        <v>11.83870300237442</v>
+        <v>12.16398286165632</v>
       </c>
       <c r="O8" t="n">
+        <v>0.1375358217082643</v>
+      </c>
+      <c r="P8" t="n">
         <v>-0.02457005868142936</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>3460745</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>3292460</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0.951373186987195</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>-0.92</v>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="n">
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="n">
         <v>1.295</v>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>[[1747368000000, 1.745], [1747972800000, 1.99], [1748577600000, 2.17], [1749182400000, 2.84], [1749787200000, 2.59], [1750392000000, 2.61], [1750996800000, 2.81], [1751601600000, 3.19], [1752206400000, 4.18], [1752811200000, 4.63], [1753416000000, 4.95], [1754020800000, 3.91], [1754625600000, 3.0], [1755230400000, 3.33], [1755835200000, 3.58], [1756440000000, 3.06], [1757044800000, 2.96], [1757649600000, 3.22], [1758254400000, 3.09], [1758859200000, 3.34], [1759464000000, 3.96], [1760068800000, 4.32], [1760673600000, 5.03], [1761278400000, 5.59], [1761883200000, 4.95], [1762491600000, 4.09], [1763096400000, 3.99], [1763701200000, 3.29], [1764306000000, 4.3], [1764910800000, 5.13], [1765515600000, 5.14], [1766120400000, 4.36], [1766725200000, 4.41], [1767330000000, 4.19], [1767934800000, 4.56], [1768539600000, 4.58], [1769144400000, 4.83], [1769749200000, 4.43], [1770354000000, 3.93], [1770958800000, 3.85], [1771563600000, 4.01], [1772168400000, 4.21], [1772773200000, 3.15], [1773374400000, 3.36], [1773979200000, 3.11], [1774584000000, 2.77], [1775188800000, 3.2], [1775793600000, 3.09], [1776398400000, 3.52], [1777003200000, 3.29], [1777608000000, 3.27], [1778212800000, 3.51], [1778817600000, 3.07], [1779422400000, 3.07], [1780027200000, 3.3], [1780632000000, 2.68], [1781236800000, 2.68], [1781841600000, 3.15], [1782446400000, 3.42], [1783051200000, 4.01], [1783656000000, 3.97]]</t>
         </is>
@@ -1140,7 +1166,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>982095040</v>
+        <v>998078464</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1157,34 +1183,37 @@
         <v>4.420000076293945</v>
       </c>
       <c r="L9" t="n">
-        <v>0.06569345479222655</v>
+        <v>0.04285718786473258</v>
       </c>
       <c r="M9" t="n">
-        <v>4.075333282316906</v>
+        <v>2.982030723977402</v>
       </c>
       <c r="N9" t="n">
-        <v>2.326178889585617</v>
+        <v>1.377238641190348</v>
       </c>
       <c r="O9" t="n">
+        <v>0.04285718786473258</v>
+      </c>
+      <c r="P9" t="n">
         <v>-0.05194800369332064</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>101836</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>37720</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>0.3703994658077693</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>-0.62</v>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="n">
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="n">
         <v>1.68</v>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>[[1747368000000, 4.06], [1747972800000, 4.73], [1748577600000, 3.97], [1749182400000, 4.05], [1749787200000, 4.27], [1750392000000, 3.76], [1750996800000, 4.16], [1751601600000, 4.2], [1752206400000, 4.07], [1752811200000, 4.26], [1753416000000, 4.26], [1754020800000, 4.02], [1754625600000, 3.93], [1755230400000, 3.76], [1755835200000, 3.64], [1756440000000, 3.5], [1757044800000, 3.48], [1757649600000, 3.47], [1758254400000, 3.64], [1758859200000, 3.48], [1759464000000, 4.01], [1760068800000, 3.87], [1760673600000, 3.88], [1761278400000, 4.1], [1761883200000, 4.07], [1762491600000, 3.08], [1763096400000, 3.02], [1763701200000, 2.97], [1764306000000, 3.33], [1764910800000, 3.12], [1765515600000, 3.01], [1766120400000, 2.95], [1766725200000, 3.11], [1767330000000, 3.18], [1767934800000, 3.66], [1768539600000, 3.61], [1769144400000, 3.61], [1769749200000, 3.65], [1770354000000, 3.53], [1770958800000, 3.51], [1771563600000, 3.53], [1772168400000, 3.4], [1772773200000, 3.07], [1773374400000, 2.31], [1773979200000, 2.43], [1774584000000, 2.42], [1775188800000, 2.59], [1775793600000, 2.63], [1776398400000, 3.26], [1777003200000, 3.15], [1777608000000, 3.09], [1778212800000, 3.07], [1778817600000, 2.7], [1779422400000, 3.03], [1780027200000, 3.07], [1780632000000, 2.8], [1781236800000, 2.72], [1781841600000, 2.56], [1782446400000, 2.74], [1783051200000, 2.9], [1783656000000, 2.92]]</t>
         </is>
@@ -1220,7 +1249,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>329073760</v>
+        <v>320348288</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1237,34 +1266,37 @@
         <v>2.089999914169312</v>
       </c>
       <c r="L10" t="n">
-        <v>0.03906255675247072</v>
+        <v>-0.01481480042466765</v>
       </c>
       <c r="M10" t="n">
-        <v>1.412243478341324</v>
+        <v>-2.785168104962621</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.3369109143899651</v>
+        <v>-4.389960187749676</v>
       </c>
       <c r="O10" t="n">
+        <v>0.01526725267893325</v>
+      </c>
+      <c r="P10" t="n">
         <v>-0.2035927682075241</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>1403298</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>935260</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0.6664728375583804</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>-0.29</v>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="n">
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="n">
         <v>6.893</v>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>[[1747368000000, 0.46], [1747972800000, 0.7], [1748577600000, 0.66], [1749182400000, 0.68], [1749787200000, 0.81], [1750392000000, 0.95], [1750996800000, 0.94], [1751601600000, 1.01], [1752206400000, 1.03], [1752811200000, 0.96], [1753416000000, 1.13], [1754020800000, 0.99], [1754625600000, 0.98], [1755230400000, 1.2], [1755835200000, 1.2], [1756440000000, 1.17], [1757044800000, 1.22], [1757649600000, 1.34], [1758254400000, 1.53], [1758859200000, 1.71], [1759464000000, 1.69], [1760068800000, 1.66], [1760673600000, 1.65], [1761278400000, 1.7], [1761883200000, 1.92], [1762491600000, 1.76], [1763096400000, 1.88], [1763701200000, 1.74], [1764306000000, 1.76], [1764910800000, 1.72], [1765515600000, 1.66], [1766120400000, 1.68], [1766725200000, 1.65], [1767330000000, 1.64], [1767934800000, 1.71], [1768539600000, 1.7], [1769144400000, 1.61], [1769749200000, 1.48], [1770354000000, 1.7], [1770958800000, 1.66], [1771563600000, 1.81], [1772168400000, 1.92], [1772773200000, 1.85], [1773374400000, 1.61], [1773979200000, 1.45], [1774584000000, 1.49], [1775188800000, 1.57], [1775793600000, 1.48], [1776398400000, 1.71], [1777003200000, 1.55], [1777608000000, 1.53], [1778212800000, 1.37], [1778817600000, 1.25], [1779422400000, 1.3], [1780027200000, 1.33], [1780632000000, 1.19], [1781236800000, 1.27], [1781841600000, 1.21], [1782446400000, 1.28], [1783051200000, 1.35], [1783656000000, 1.33]]</t>
         </is>
@@ -1300,7 +1332,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>204871072</v>
+        <v>194867488</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1317,34 +1349,37 @@
         <v>2.839999914169312</v>
       </c>
       <c r="L11" t="n">
-        <v>0.087447160776007</v>
+        <v>-0.03504380008766883</v>
       </c>
       <c r="M11" t="n">
-        <v>6.250703880694952</v>
+        <v>-4.808068071262738</v>
       </c>
       <c r="N11" t="n">
-        <v>4.501549487963663</v>
+        <v>-6.412860154049794</v>
       </c>
       <c r="O11" t="n">
+        <v>-0.01153838982478372</v>
+      </c>
+      <c r="P11" t="n">
         <v>-0.1977107103217441</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>9229285</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>18299380</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>1.982751643274641</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>-0.63</v>
       </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="n">
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
         <v>3.929</v>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>[[1747368000000, 2.24], [1747972800000, 2.53], [1748577600000, 2.67], [1749182400000, 2.59], [1749787200000, 2.37], [1750392000000, 2.31], [1750996800000, 2.12], [1751601600000, 2.28], [1752206400000, 2.31], [1752811200000, 2.33], [1753416000000, 2.53], [1754020800000, 2.28], [1754625600000, 2.48], [1755230400000, 1.88], [1755835200000, 1.58], [1756440000000, 1.55], [1757044800000, 1.43], [1757649600000, 1.47], [1758254400000, 1.86], [1758859200000, 1.73], [1759464000000, 2.1], [1760068800000, 1.56], [1760673600000, 1.72], [1761278400000, 1.71], [1761883200000, 1.67], [1762491600000, 1.33], [1763096400000, 1.23], [1763701200000, 1.22], [1764306000000, 1.35], [1764910800000, 1.23], [1765515600000, 1.31], [1766120400000, 1.11], [1766725200000, 1.07], [1767330000000, 0.975], [1767934800000, 1.17], [1768539600000, 1.11], [1769144400000, 1.05], [1769749200000, 0.998], [1770354000000, 0.938], [1770958800000, 1.01], [1771563600000, 1.13], [1772168400000, 1.115], [1772773200000, 1.11], [1773374400000, 1.16], [1773979200000, 0.783], [1774584000000, 0.676], [1775188800000, 0.642], [1775793600000, 0.645], [1776398400000, 0.71], [1777003200000, 0.7], [1777608000000, 0.855], [1778212800000, 1.06], [1778817600000, 0.93], [1779422400000, 1.05], [1780027200000, 1.3], [1780632000000, 1.35], [1781236800000, 1.055], [1781841600000, 0.924], [1782446400000, 0.709], [1783051200000, 0.71], [1783656000000, 0.771]]</t>
         </is>
@@ -1380,7 +1415,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>5967351</v>
+        <v>6232882</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1397,34 +1432,37 @@
         <v>55</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2545454260841</v>
+        <v>0.2297029658563345</v>
       </c>
       <c r="M12" t="n">
-        <v>22.96053041150425</v>
+        <v>21.6666085231376</v>
       </c>
       <c r="N12" t="n">
-        <v>21.21137601877297</v>
+        <v>20.06181644035054</v>
       </c>
       <c r="O12" t="n">
+        <v>0.1965317905798245</v>
+      </c>
+      <c r="P12" t="n">
         <v>-0.6451428617749895</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>696828</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>312880</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>0.4490060674944176</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>-5.06</v>
       </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="n">
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
         <v>5.607</v>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>[[1747368000000, 12.35], [1747972800000, 13.75], [1748577600000, 16.7], [1749182400000, 14.4], [1749787200000, 14.6], [1750392000000, 13.2], [1750996800000, 11.15], [1751601600000, 13.0], [1752206400000, 13.85], [1752811200000, 13.85], [1753416000000, 13.6], [1754020800000, 11.55], [1754625600000, 10.7], [1755230400000, 10.6], [1755835200000, 8.4], [1756440000000, 8.2], [1757044800000, 11.5], [1757649600000, 14.6], [1758254400000, 11.65], [1758859200000, 8.95], [1759464000000, 9.6], [1760068800000, 10.25], [1760673600000, 18.15], [1761278400000, 9.61], [1761883200000, 5.77], [1762491600000, 4.21], [1763096400000, 4.43], [1763701200000, 3.0], [1764306000000, 2.96], [1764910800000, 3.36], [1765515600000, 2.84], [1766120400000, 2.13], [1766725200000, 1.79], [1767330000000, 1.79], [1767934800000, 2.2], [1768539600000, 3.0], [1769144400000, 2.84], [1769749200000, 2.66], [1770354000000, 2.2], [1770958800000, 2.02], [1771563600000, 1.78], [1772168400000, 2.0], [1772773200000, 1.95], [1773374400000, 2.01], [1773979200000, 1.88], [1774584000000, 1.82], [1775188800000, 1.54], [1775793600000, 1.15], [1776398400000, 1.3], [1777003200000, 1.02], [1777608000000, 0.918], [1778212800000, 0.87], [1778817600000, 0.83], [1779422400000, 0.821], [1780027200000, 0.78], [1780632000000, 0.647], [1781236800000, 0.64], [1781841600000, 0.592], [1782446400000, 0.495], [1783051200000, 0.576], [1783656000000, 0.621]]</t>
         </is>
@@ -1460,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>436458656</v>
+        <v>418423168</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1477,34 +1515,37 @@
         <v>3.039999961853027</v>
       </c>
       <c r="L13" t="n">
-        <v>0.03448282949422898</v>
+        <v>-0.004149373488428698</v>
       </c>
       <c r="M13" t="n">
-        <v>0.9542707525171501</v>
+        <v>-1.718625411338726</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.794883640214139</v>
+        <v>-3.32341749412578</v>
       </c>
       <c r="O13" t="n">
+        <v>-0.02040814340536656</v>
+      </c>
+      <c r="P13" t="n">
         <v>1.412060385794805</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>1307175</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>2087760</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>1.597154168340123</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>-1.14</v>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="n">
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
         <v>10.249</v>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>[[1747368000000, 0.56], [1747972800000, 0.559], [1748577600000, 0.53], [1749182400000, 0.616], [1749787200000, 0.575], [1750392000000, 0.582], [1750996800000, 0.519], [1751601600000, 0.555], [1752206400000, 0.6], [1752811200000, 0.581], [1753416000000, 0.626], [1754020800000, 0.532], [1754625600000, 0.507], [1755230400000, 0.562], [1755835200000, 0.541], [1756440000000, 0.492], [1757044800000, 0.505], [1757649600000, 0.501], [1758254400000, 0.477], [1758859200000, 0.509], [1759464000000, 0.513], [1760068800000, 0.569], [1760673600000, 0.542], [1761278400000, 0.577], [1761883200000, 0.583], [1762491600000, 0.535], [1763096400000, 0.472], [1763701200000, 0.49], [1764306000000, 0.545], [1764910800000, 0.526], [1765515600000, 0.558], [1766120400000, 0.9], [1766725200000, 1.085], [1767330000000, 0.995], [1767934800000, 1.94], [1768539600000, 2.17], [1769144400000, 2.42], [1769749200000, 1.9], [1770354000000, 1.7], [1770958800000, 1.75], [1771563600000, 2.06], [1772168400000, 2.32], [1772773200000, 2.56], [1773374400000, 2.34], [1773979200000, 2.42], [1774584000000, 2.02], [1775188800000, 2.13], [1775793600000, 2.25], [1776398400000, 2.6], [1777003200000, 2.22], [1777608000000, 2.31], [1778212800000, 2.29], [1778817600000, 2.34], [1779422400000, 2.26], [1780027200000, 2.45], [1780632000000, 2.13], [1781236800000, 2.25], [1781841600000, 2.29], [1782446400000, 2.32], [1783051200000, 2.43], [1783656000000, 2.4]]</t>
         </is>
@@ -1540,11 +1581,11 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>290563552</v>
+        <v>303562464</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Micro-cap</t>
+          <t>Small-cap</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1557,34 +1598,37 @@
         <v>6.599999904632568</v>
       </c>
       <c r="L14" t="n">
-        <v>0.03157898039038542</v>
+        <v>0.005128200112166859</v>
       </c>
       <c r="M14" t="n">
-        <v>0.6638858421327942</v>
+        <v>-0.7908680512791699</v>
       </c>
       <c r="N14" t="n">
-        <v>-1.085268550598495</v>
+        <v>-2.395660134066224</v>
       </c>
       <c r="O14" t="n">
+        <v>0.005128200112166859</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.04812835997278464</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>784064</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>457800</v>
       </c>
-      <c r="R14" t="n">
+      <c r="S14" t="n">
         <v>0.5838809076810056</v>
       </c>
-      <c r="S14" t="n">
-        <v>-0.58</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="n">
+      <c r="T14" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
         <v>11.447</v>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>[[1747368000000, 1.85], [1747972800000, 1.81], [1748577600000, 1.93], [1749182400000, 1.81], [1749787200000, 1.71], [1750392000000, 1.79], [1750996800000, 1.69], [1751601600000, 1.72], [1752206400000, 2.6], [1752811200000, 2.57], [1753416000000, 2.55], [1754020800000, 2.23], [1754625600000, 2.2], [1755230400000, 2.22], [1755835200000, 2.195], [1756440000000, 2.08], [1757044800000, 2.27], [1757649600000, 2.12], [1758254400000, 2.47], [1758859200000, 2.01], [1759464000000, 2.06], [1760068800000, 2.29], [1760673600000, 2.51], [1761278400000, 3.03], [1761883200000, 3.25], [1762491600000, 3.2], [1763096400000, 3.24], [1763701200000, 3.95], [1764306000000, 3.95], [1764910800000, 3.98], [1765515600000, 3.81], [1766120400000, 3.99], [1766725200000, 3.78], [1767330000000, 3.77], [1767934800000, 3.68], [1768539600000, 3.98], [1769144400000, 4.04], [1769749200000, 4.39], [1770354000000, 4.17], [1770958800000, 3.85], [1771563600000, 3.57], [1772168400000, 4.1], [1772773200000, 3.79], [1773374400000, 4.15], [1773979200000, 3.75], [1774584000000, 3.85], [1775188800000, 3.88], [1775793600000, 3.75], [1776398400000, 3.85], [1777003200000, 3.52], [1777608000000, 3.47], [1778212800000, 4.11], [1778817600000, 3.7], [1779422400000, 3.9], [1780027200000, 3.6], [1780632000000, 3.38], [1781236800000, 3.33], [1781841600000, 4.0], [1782446400000, 3.8], [1783051200000, 3.92], [1783656000000, 3.92]]</t>
         </is>
@@ -1620,7 +1664,7 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>35120752</v>
+        <v>33987824</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1637,34 +1681,37 @@
         <v>0.1599999964237213</v>
       </c>
       <c r="L15" t="n">
+        <v>-0.09999997764825852</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-11.30368582732171</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-12.90847791010876</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-0.09999997764825852</v>
+      </c>
+      <c r="P15" t="n">
         <v>0</v>
       </c>
-      <c r="M15" t="n">
-        <v>-2.494012196905748</v>
-      </c>
-      <c r="N15" t="n">
-        <v>-4.243166589637037</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>35025.27472527473</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>7840</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>0.2238383584852383</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>-0.03</v>
       </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="n">
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
         <v>0.139</v>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>[[1747368000000, 0.15], [1747972800000, 0.14], [1748577600000, 0.13], [1749182400000, 0.12], [1749787200000, 0.13], [1750392000000, 0.12], [1750996800000, 0.12], [1751601600000, 0.11], [1752206400000, 0.12], [1752811200000, 0.12], [1753416000000, 0.14], [1754020800000, 0.14], [1754625600000, 0.15], [1755230400000, 0.15], [1755835200000, 0.13], [1756440000000, 0.13], [1757044800000, 0.13], [1757649600000, 0.13], [1758254400000, 0.13], [1758859200000, 0.13], [1759464000000, 0.14], [1760068800000, 0.13], [1760673600000, 0.12], [1761278400000, 0.12], [1761883200000, 0.11], [1762491600000, 0.11], [1763096400000, 0.1], [1763701200000, 0.1], [1764306000000, 0.11], [1764910800000, 0.1], [1765515600000, 0.1], [1766120400000, 0.09], [1766725200000, 0.1], [1767330000000, 0.09], [1767934800000, 0.11], [1768539600000, 0.12], [1769144400000, 0.12], [1769749200000, 0.12], [1770354000000, 0.11], [1770958800000, 0.1], [1771563600000, 0.1], [1772168400000, 0.1], [1772773200000, 0.12], [1773374400000, 0.12], [1773979200000, 0.11], [1774584000000, 0.12], [1775188800000, 0.11], [1775793600000, 0.14], [1776398400000, 0.14], [1777003200000, 0.13], [1777608000000, 0.13], [1778212800000, 0.12], [1778817600000, 0.12], [1779422400000, 0.11], [1780027200000, 0.11], [1780632000000, 0.12], [1781236800000, 0.11], [1781841600000, 0.11], [1782446400000, 0.09], [1783051200000, 0.09], [1783656000000, 0.09]]</t>
         </is>
@@ -1700,7 +1747,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>21804678</v>
+        <v>22572956</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1717,34 +1764,37 @@
         <v>28.03000068664551</v>
       </c>
       <c r="L16" t="n">
-        <v>0.07280215902427067</v>
+        <v>0.05826555849195914</v>
       </c>
       <c r="M16" t="n">
-        <v>4.786203705521319</v>
+        <v>4.522867786700058</v>
       </c>
       <c r="N16" t="n">
-        <v>3.03704931279003</v>
+        <v>2.918075703913003</v>
       </c>
       <c r="O16" t="n">
+        <v>0.06693985787256507</v>
+      </c>
+      <c r="P16" t="n">
         <v>1.055263168626875</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>42221</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>57280</v>
       </c>
-      <c r="R16" t="n">
+      <c r="S16" t="n">
         <v>1.356670850998318</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>-2.16</v>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="n">
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
         <v>0.759</v>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>[[1747368000000, 16.16], [1747972800000, 18.5], [1748577600000, 22.0], [1749182400000, 23.0], [1749787200000, 22.8], [1750392000000, 24.1], [1750996800000, 27.9], [1751601600000, 24.4], [1752206400000, 21.0], [1752811200000, 22.2], [1753416000000, 19.8], [1754020800000, 18.0], [1754625600000, 21.4], [1755230400000, 25.1], [1755835200000, 26.3], [1756440000000, 21.2], [1757044800000, 19.6], [1757649600000, 21.5], [1758254400000, 20.4], [1758859200000, 21.9], [1759464000000, 19.95], [1760068800000, 17.6], [1760673600000, 16.5], [1761278400000, 13.0], [1761883200000, 7.29], [1762491600000, 4.01], [1763096400000, 3.49], [1763701200000, 3.27], [1764306000000, 4.01], [1764910800000, 3.64], [1765515600000, 2.91], [1766120400000, 2.6], [1766725200000, 2.5], [1767330000000, 2.09], [1767934800000, 2.19], [1768539600000, 2.36], [1769144400000, 2.67], [1769749200000, 2.6], [1770354000000, 2.77], [1770958800000, 2.77], [1771563600000, 2.7], [1772168400000, 2.9], [1772773200000, 2.77], [1773374400000, 2.74], [1773979200000, 2.37], [1774584000000, 2.22], [1775188800000, 2.255], [1775793600000, 2.49], [1776398400000, 2.66], [1777003200000, 4.66], [1777608000000, 3.85], [1778212800000, 3.36], [1778817600000, 3.21], [1779422400000, 3.16], [1780027200000, 3.52], [1780632000000, 2.93], [1781236800000, 3.23], [1781841600000, 3.31], [1782446400000, 3.64], [1783051200000, 3.85], [1783656000000, 3.905]]</t>
         </is>
@@ -1777,10 +1827,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.1037318632006645</v>
+        <v>0.1037318603586439</v>
       </c>
       <c r="G17" t="n">
-        <v>4901889.028582871</v>
+        <v>5129883.639729005</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1788,47 +1838,50 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>3.713600623442659</v>
+        <v>3.713600521698321</v>
       </c>
       <c r="J17" t="n">
-        <v>0.7771519663565698</v>
+        <v>0.7771519506376539</v>
       </c>
       <c r="K17" t="n">
-        <v>7.226800590387938</v>
+        <v>7.226800500286398</v>
       </c>
       <c r="L17" t="n">
-        <v>0.2819493734216099</v>
+        <v>0.2819493239565563</v>
       </c>
       <c r="M17" t="n">
-        <v>25.70092514525524</v>
+        <v>26.89124433315977</v>
       </c>
       <c r="N17" t="n">
-        <v>23.95177075252395</v>
+        <v>25.28645225037272</v>
       </c>
       <c r="O17" t="n">
-        <v>2.407291740743238</v>
+        <v>0.1938795044022277</v>
       </c>
       <c r="P17" t="n">
+        <v>2.407291589354331</v>
+      </c>
+      <c r="Q17" t="n">
         <v>16342.81</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>6195.2</v>
       </c>
-      <c r="R17" t="n">
+      <c r="S17" t="n">
         <v>0.3790780165712017</v>
       </c>
-      <c r="S17" t="n">
-        <v>678.84</v>
-      </c>
       <c r="T17" t="n">
-        <v>0.05067468</v>
+        <v>678.85</v>
       </c>
       <c r="U17" t="n">
+        <v>0.053030863</v>
+      </c>
+      <c r="V17" t="n">
         <v>1.334</v>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>[[1747346400000, 1.0687], [1747951200000, 1.1621], [1748556000000, 1.1626], [1749160800000, 1.2008], [1749765600000, 1.1768], [1750370400000, 1.006], [1750975200000, 0.9466], [1751580000000, 0.8467], [1752184800000, 0.8265], [1752789600000, 0.8636], [1753394400000, 1.1127], [1753999200000, 1.2162], [1754604000000, 1.1408], [1755208800000, 1.1272], [1755813600000, 1.0402], [1756418400000, 1.055], [1757023200000, 1.3646], [1757628000000, 1.4289], [1758232800000, 1.5732], [1758837600000, 1.9655], [1759442400000, 1.8736], [1760047200000, 1.6471], [1760652000000, 1.455], [1761256800000, 1.3865], [1761865200000, 1.3883], [1762470000000, 1.2959], [1763074800000, 1.3823], [1763679600000, 1.1954], [1764284400000, 1.0665], [1764889200000, 1.1248], [1765494000000, 1.1999], [1766098800000, 1.196], [1766703600000, 1.2245], [1767308400000, 1.0882], [1767913200000, 1.1392], [1768518000000, 1.1614], [1769122800000, 0.972], [1769727600000, 0.9656], [1770332400000, 1.0436], [1770937200000, 1.0366], [1771542000000, 1.2134], [1772146800000, 1.4478], [1772751600000, 1.1712], [1773356400000, 1.1773], [1773961200000, 1.3244], [1774566000000, 1.1463], [1775167200000, 1.5204], [1775772000000, 1.4812], [1776376800000, 1.534], [1776981600000, 1.4422], [1777586400000, 1.5315], [1778191200000, 3.6003], [1778796000000, 3.6377], [1779400800000, 3.6951], [1780005600000, 5.8384], [1780610400000, 4.971], [1781215200000, 4.1092], [1781820000000, 3.6493], [1782424800000, 2.8746], [1783029600000, 3.511], [1783634400000, 3.7136]]</t>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>[[1747346400000, 1.0687], [1747951200000, 1.1621], [1748556000000, 1.1626], [1749160800000, 1.2008], [1749765600000, 1.1768], [1750370400000, 1.006], [1750975200000, 0.9466], [1751580000000, 0.8467], [1752184800000, 0.8265], [1752789600000, 0.8636], [1753394400000, 1.1127], [1753999200000, 1.2162], [1754604000000, 1.1408], [1755208800000, 1.1272], [1755813600000, 1.0402], [1756418400000, 1.055], [1757023200000, 1.3646], [1757628000000, 1.4289], [1758232800000, 1.5732], [1758837600000, 1.9656], [1759442400000, 1.8736], [1760047200000, 1.6471], [1760652000000, 1.455], [1761256800000, 1.3865], [1761865200000, 1.3883], [1762470000000, 1.2959], [1763074800000, 1.3823], [1763679600000, 1.1954], [1764284400000, 1.0665], [1764889200000, 1.1248], [1765494000000, 1.1999], [1766098800000, 1.196], [1766703600000, 1.2245], [1767308400000, 1.0882], [1767913200000, 1.1392], [1768518000000, 1.1614], [1769122800000, 0.972], [1769727600000, 0.9656], [1770332400000, 1.0436], [1770937200000, 1.0366], [1771542000000, 1.2134], [1772146800000, 1.4478], [1772751600000, 1.1712], [1773356400000, 1.1773], [1773961200000, 1.3244], [1774566000000, 1.1463], [1775167200000, 1.5204], [1775772000000, 1.4812], [1776376800000, 1.534], [1776981600000, 1.4422], [1777586400000, 1.5315], [1778191200000, 3.6003], [1778796000000, 3.6377], [1779400800000, 3.6951], [1780005600000, 5.8384], [1780610400000, 4.971], [1781215200000, 4.1092], [1781820000000, 3.6493], [1782424800000, 2.8746], [1783029600000, 3.511], [1783634400000, 3.7136]]</t>
         </is>
       </c>
     </row>
@@ -1859,10 +1912,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.1037318632006645</v>
+        <v>0.1037318603586439</v>
       </c>
       <c r="G18" t="n">
-        <v>11670549.11514848</v>
+        <v>13218919.42106998</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1870,43 +1923,46 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>0.1037318632006645</v>
+        <v>0.1037318603586439</v>
       </c>
       <c r="J18" t="n">
-        <v>0.06640735739870784</v>
+        <v>0.06640735892066295</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2004888715578534</v>
+        <v>0.200488872986427</v>
       </c>
       <c r="L18" t="n">
-        <v>0.01589912203100141</v>
+        <v>0.01589908283171182</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.9040999938056071</v>
+        <v>0.2862202206753262</v>
       </c>
       <c r="N18" t="n">
-        <v>-2.653254386536896</v>
+        <v>-1.318571862111728</v>
       </c>
       <c r="O18" t="n">
-        <v>0.3019938190061535</v>
+        <v>0.07255318297063673</v>
       </c>
       <c r="P18" t="n">
+        <v>0.3019937611574468</v>
+      </c>
+      <c r="Q18" t="n">
         <v>426816.02</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>831253.4</v>
       </c>
-      <c r="R18" t="n">
+      <c r="S18" t="n">
         <v>1.947568416012126</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>-0.43</v>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="n">
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="n">
         <v>4.898</v>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>[[1747346400000, 0.1062], [1747951200000, 0.1069], [1748556000000, 0.1131], [1749160800000, 0.1126], [1749765600000, 0.1088], [1750370400000, 0.1034], [1750975200000, 0.1058], [1751580000000, 0.1129], [1752184800000, 0.1063], [1752789600000, 0.1075], [1753394400000, 0.1329], [1753999200000, 0.1198], [1754604000000, 0.1269], [1755208800000, 0.1219], [1755813600000, 0.1192], [1756418400000, 0.1234], [1757023200000, 0.114], [1757628000000, 0.1154], [1758232800000, 0.1068], [1758837600000, 0.102], [1759442400000, 0.1039], [1760047200000, 0.0975], [1760652000000, 0.0977], [1761256800000, 0.0991], [1761865200000, 0.0958], [1762470000000, 0.0857], [1763074800000, 0.0844], [1763679600000, 0.0839], [1764284400000, 0.0813], [1764889200000, 0.078], [1765494000000, 0.0738], [1766098800000, 0.072], [1766703600000, 0.0754], [1767308400000, 0.0764], [1767913200000, 0.0745], [1768518000000, 0.1389], [1769122800000, 0.1522], [1769727600000, 0.1477], [1770332400000, 0.1754], [1770937200000, 0.1609], [1771542000000, 0.1699], [1772146800000, 0.1558], [1772751600000, 0.1438], [1773356400000, 0.1391], [1773961200000, 0.129], [1774566000000, 0.1344], [1775167200000, 0.1291], [1775772000000, 0.1484], [1776376800000, 0.1425], [1776981600000, 0.1264], [1777586400000, 0.1184], [1778191200000, 0.1326], [1778796000000, 0.1164], [1779400800000, 0.1221], [1780005600000, 0.1351], [1780610400000, 0.1184], [1781215200000, 0.1123], [1781820000000, 0.1108], [1782424800000, 0.1027], [1783029600000, 0.0981], [1783634400000, 0.1037]]</t>
         </is>
@@ -1942,7 +1998,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>1694332416</v>
+        <v>1678818432</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1959,34 +2015,37 @@
         <v>40.71500015258789</v>
       </c>
       <c r="L19" t="n">
-        <v>0.03432647027522462</v>
+        <v>0.04996714181300077</v>
       </c>
       <c r="M19" t="n">
-        <v>0.9386348306167136</v>
+        <v>3.693026118804221</v>
       </c>
       <c r="N19" t="n">
-        <v>-0.8105195621145755</v>
+        <v>2.088234036017167</v>
       </c>
       <c r="O19" t="n">
+        <v>0.005984268789216207</v>
+      </c>
+      <c r="P19" t="n">
         <v>-0.07980405138224811</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>434591</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>638000</v>
       </c>
-      <c r="R19" t="n">
+      <c r="S19" t="n">
         <v>1.468046968298929</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="n">
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="n">
         <v>4.181</v>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>[[1747368000000, 30.37], [1747972800000, 31.16], [1748577600000, 36.6], [1749182400000, 37.25], [1749787200000, 34.68], [1750392000000, 31.34], [1750996800000, 31.12], [1751601600000, 33.02], [1752206400000, 35.02], [1752811200000, 36.31], [1753416000000, 35.17], [1754020800000, 32.99], [1754625600000, 31.97], [1755230400000, 32.88], [1755835200000, 32.93], [1756440000000, 32.22], [1757044800000, 37.2], [1757649600000, 35.24], [1758254400000, 32.6], [1758859200000, 34.02], [1759464000000, 34.21], [1760068800000, 32.4], [1760673600000, 33.56], [1761278400000, 33.105], [1761883200000, 33.09], [1762491600000, 33.5], [1763096400000, 35.95], [1763701200000, 39.35], [1764306000000, 39.5], [1764910800000, 38.78], [1765515600000, 36.8], [1766120400000, 36.01], [1766725200000, 36.13], [1767330000000, 33.78], [1767934800000, 33.0], [1768539600000, 33.35], [1769144400000, 35.11], [1769749200000, 32.55], [1770354000000, 31.98], [1770958800000, 32.28], [1771563600000, 32.68], [1772168400000, 32.3], [1772773200000, 32.94], [1773374400000, 30.86], [1773979200000, 29.91], [1774584000000, 29.44], [1775188800000, 30.83], [1775793600000, 31.05], [1776398400000, 31.45], [1777003200000, 29.3], [1777608000000, 28.16], [1778212800000, 29.58], [1778817600000, 28.05], [1779422400000, 28.83], [1780027200000, 28.89], [1780632000000, 28.29], [1781236800000, 28.96], [1781841600000, 28.6], [1782446400000, 30.88], [1783051200000, 32.5], [1783656000000, 31.94]]</t>
         </is>
@@ -2022,7 +2081,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>3668573</v>
+        <v>3511834</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2039,34 +2098,37 @@
         <v>6.25</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.0416667246156246</v>
+        <v>0.4194026293138329</v>
       </c>
       <c r="M20" t="n">
-        <v>-6.660684658468208</v>
+        <v>40.63657486888743</v>
       </c>
       <c r="N20" t="n">
-        <v>-8.409839051199498</v>
+        <v>39.03178278610038</v>
       </c>
       <c r="O20" t="n">
+        <v>-0.2068965942482588</v>
+      </c>
+      <c r="P20" t="n">
         <v>-0.4132653297061272</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>2039520</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>39666180</v>
       </c>
-      <c r="R20" t="n">
+      <c r="S20" t="n">
         <v>19.44878206636856</v>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>-2.07</v>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="n">
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
         <v>19.694</v>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>[[1747368000000, 2.02], [1747972800000, 2.02], [1748577600000, 2.18], [1749182400000, 2.3943], [1749787200000, 2.18], [1750392000000, 2.47], [1750996800000, 2.65], [1751601600000, 2.67], [1752206400000, 2.91], [1752811200000, 2.77], [1753416000000, 2.7099], [1754020800000, 2.87], [1754625600000, 3.33], [1755230400000, 3.12], [1755835200000, 3.19], [1756440000000, 3.18], [1757044800000, 3.31], [1757649600000, 3.5], [1758254400000, 3.51], [1758859200000, 3.305], [1759464000000, 3.235], [1760068800000, 3.33], [1760673600000, 3.59], [1761278400000, 4.88], [1761883200000, 3.17], [1762491600000, 3.02], [1763096400000, 3.15], [1763701200000, 2.73], [1764306000000, 2.69], [1764910800000, 2.34], [1765515600000, 2.15], [1766120400000, 2.11], [1766725200000, 2.1], [1767330000000, 1.97], [1767934800000, 2.25], [1768539600000, 2.0], [1769144400000, 2.1], [1769749200000, 2.02], [1770354000000, 1.93], [1770958800000, 1.86], [1771563600000, 1.9], [1772168400000, 1.81], [1772773200000, 1.88], [1773374400000, 1.88], [1773979200000, 1.84], [1774584000000, 1.97], [1775188800000, 2.0534], [1775793600000, 2.14], [1776398400000, 2.47], [1777003200000, 2.3], [1777608000000, 2.24], [1778212800000, 2.31], [1778817600000, 2.24], [1779422400000, 2.39], [1780027200000, 2.25], [1780632000000, 2.06], [1781236800000, 2.17], [1781841600000, 2.23], [1782446400000, 1.2], [1783051200000, 1.21], [1783656000000, 1.15]]</t>
         </is>
@@ -2102,7 +2164,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>326504512</v>
+        <v>308751296</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2119,34 +2181,37 @@
         <v>4.599999904632568</v>
       </c>
       <c r="L21" t="n">
-        <v>0.05026456578268257</v>
+        <v>0.02319585348318465</v>
       </c>
       <c r="M21" t="n">
-        <v>2.532444381362509</v>
+        <v>1.015897285822609</v>
       </c>
       <c r="N21" t="n">
-        <v>0.7832899886312195</v>
+        <v>-0.5888947969644454</v>
       </c>
       <c r="O21" t="n">
+        <v>0.007614205825909215</v>
+      </c>
+      <c r="P21" t="n">
         <v>1.629139108399771</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>1427144</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>1606880</v>
       </c>
-      <c r="R21" t="n">
+      <c r="S21" t="n">
         <v>1.125941040287455</v>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>-0.77</v>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="n">
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
         <v>8.439</v>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>[[1747368000000, 2.87], [1747972800000, 3.05], [1748577600000, 3.0], [1749182400000, 3.08], [1749787200000, 2.87], [1750392000000, 2.72], [1750996800000, 2.69], [1751601600000, 3.08], [1752206400000, 3.42], [1752811200000, 3.7], [1753416000000, 3.62], [1754020800000, 3.38], [1754625600000, 2.715], [1755230400000, 2.63], [1755835200000, 2.6], [1756440000000, 2.59], [1757044800000, 2.71], [1757649600000, 2.42], [1758254400000, 2.55], [1758859200000, 2.69], [1759464000000, 2.84], [1760068800000, 2.74], [1760673600000, 3.44], [1761278400000, 3.48], [1761883200000, 4.32], [1762491600000, 2.06], [1763096400000, 1.76], [1763701200000, 1.44], [1764306000000, 1.63], [1764910800000, 1.58], [1765515600000, 1.64], [1766120400000, 1.64], [1766725200000, 1.6], [1767330000000, 1.62], [1767934800000, 1.73], [1768539600000, 2.12], [1769144400000, 2.14], [1769749200000, 2.2], [1770354000000, 2.19], [1770958800000, 2.02], [1771563600000, 2.19], [1772168400000, 2.62], [1772773200000, 2.78], [1773374400000, 2.69], [1773979200000, 2.88], [1774584000000, 2.83], [1775188800000, 3.07], [1775793600000, 3.1], [1776398400000, 3.98], [1777003200000, 3.465], [1777608000000, 3.69], [1778212800000, 3.88], [1778817600000, 3.8], [1779422400000, 3.89], [1780027200000, 3.81], [1780632000000, 3.41], [1781236800000, 3.57], [1781841600000, 3.92], [1782446400000, 3.78], [1783051200000, 3.95], [1783656000000, 3.97]]</t>
         </is>
@@ -2179,10 +2244,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.143772125244141</v>
+        <v>1.143772156593257</v>
       </c>
       <c r="G22" t="n">
-        <v>86257272.8694458</v>
+        <v>88880731.70394319</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2190,43 +2255,46 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>4.838156111598437</v>
+        <v>4.838156244205199</v>
       </c>
       <c r="J22" t="n">
-        <v>4.374948659362531</v>
+        <v>4.374948656004105</v>
       </c>
       <c r="K22" t="n">
-        <v>14.38681953993705</v>
+        <v>14.38681984210267</v>
       </c>
       <c r="L22" t="n">
-        <v>0.04612324943834278</v>
+        <v>0.04612331235195488</v>
       </c>
       <c r="M22" t="n">
-        <v>2.11831274692853</v>
+        <v>3.308643172699632</v>
       </c>
       <c r="N22" t="n">
-        <v>0.369158354197241</v>
+        <v>1.703851089912578</v>
       </c>
       <c r="O22" t="n">
-        <v>-0.3852941973260497</v>
+        <v>0.02314155590565403</v>
       </c>
       <c r="P22" t="n">
+        <v>-0.3852941742109731</v>
+      </c>
+      <c r="Q22" t="n">
         <v>226317.04</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="R22" t="n">
         <v>204584.4</v>
       </c>
-      <c r="R22" t="n">
+      <c r="S22" t="n">
         <v>0.9039725864212433</v>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>-0.9</v>
       </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="n">
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
         <v>1.192</v>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>[[1747346400000, 4.8185], [1747951200000, 4.0276], [1748556000000, 4.1929], [1749160800000, 3.9745], [1749765600000, 4.1993], [1750370400000, 4.3346], [1750975200000, 4.3963], [1751580000000, 4.4496], [1752184800000, 4.4002], [1752789600000, 4.7914], [1753394400000, 8.9347], [1753999200000, 7.6539], [1754604000000, 7.8234], [1755208800000, 11.4649], [1755813600000, 10.3356], [1756418400000, 9.6723], [1757023200000, 9.3605], [1757628000000, 9.6108], [1758232800000, 8.9612], [1758837600000, 8.5138], [1759442400000, 9.0166], [1760047200000, 11.2773], [1760652000000, 11.5475], [1761256800000, 10.3633], [1761865200000, 10.0912], [1762470000000, 10.0247], [1763074800000, 10.3292], [1763679600000, 8.9739], [1764284400000, 9.3843], [1764889200000, 8.7787], [1765494000000, 8.2176], [1766098800000, 7.7038], [1766703600000, 7.5019], [1767308400000, 7.9081], [1767913200000, 6.9947], [1768518000000, 7.0235], [1769122800000, 7.664], [1769727600000, 7.6581], [1770332400000, 7.6909], [1770937200000, 7.5721], [1771542000000, 8.2384], [1772146800000, 7.908], [1772751600000, 7.3131], [1773356400000, 6.8323], [1773961200000, 6.2519], [1774566000000, 5.2658], [1775167200000, 5.378], [1775772000000, 5.5136], [1776376800000, 6.0799], [1776981600000, 5.419], [1777586400000, 5.7021], [1778191200000, 5.6147], [1778796000000, 5.7168], [1779400800000, 5.5898], [1780005600000, 5.7495], [1780610400000, 4.9702], [1781215200000, 4.9545], [1781820000000, 4.7324], [1782424800000, 4.806], [1783029600000, 5.0877], [1783634400000, 4.8382]]</t>
         </is>

</xml_diff>